<commit_message>
Move website files to root
</commit_message>
<xml_diff>
--- a/backend/upay-data.xlsx
+++ b/backend/upay-data.xlsx
@@ -471,7 +471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -908,16 +908,45 @@
         <v>2026-04-02 07:49:42</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>97vleed</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Self Awareness</v>
+      </c>
+      <c r="D16" t="str">
+        <v>IT Park</v>
+      </c>
+      <c r="E16">
+        <v>30000</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Income</v>
+      </c>
+      <c r="H16" t="str">
+        <v>admin</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2026-06-15 03:45:29</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1004,9 +1033,26 @@
         <v>2026-04-02 07:49:42</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>m9idxn9</v>
+      </c>
+      <c r="B6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Added transaction for Self Awareness – Credit ₹30000</v>
+      </c>
+      <c r="D6" t="str">
+        <v>add</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-06-15 03:45:29</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>